<commit_message>
Stakeholder Map: merge the Red Sea Utilities and Veolia Middle East AR/EN twins (reviewer decision 20 Oct); Veolia → Direct Competitors
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019KNqDdH7EHx9VVoh45Frou
</commit_message>
<xml_diff>
--- a/pipeline/twin_decisions.xlsx
+++ b/pipeline/twin_decisions.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3589,6 +3589,76 @@
       <c r="Q40" s="2" t="inlineStr">
         <is>
           <t>stated by Youssef 10 Sep 2026; kept the competitor record</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Red Sea Utilities Consortium</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>شركة مرافق البحر الاحمر المشتركة للطاقة</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>same company in English and Arabic (SWA water-sector chart, Oct 2026)</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Merge → keep A</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Same company: Red Sea Utilities Co. (RSG subsidiary, Umluj) — SWA desalination licence and MWAN sorting/trading licence. Decided 20 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Veolia Middle East Environmental Services</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>فيوليا ميديل ايست للخدمات البيئية</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>same company in English and Arabic (SWA water-sector chart, Oct 2026)</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Merge → keep A</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Same company: Veolia Middle East, Jubail — MWAN hazardous-waste treatment licence (thermal oxidation, 384 t/day). Direct competitor. Decided 20 Oct 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>